<commit_message>
week3-update sql_decomposition.xlsx for task 2
</commit_message>
<xml_diff>
--- a/week 3/task2/sql_decomposition.xlsx
+++ b/week 3/task2/sql_decomposition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="172">
   <si>
     <t xml:space="preserve">question</t>
   </si>
@@ -113,6 +113,9 @@
   </si>
   <si>
     <t xml:space="preserve">Retrieve product names and prices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">productName, buyPrice</t>
   </si>
   <si>
     <t xml:space="preserve">Get customer names and cities</t>
@@ -667,27 +670,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1122,7 +1125,9 @@
       <c r="C9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="6"/>
+      <c r="D9" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="E9" s="6" t="s">
         <v>10</v>
       </c>
@@ -1132,16 +1137,16 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>10</v>
@@ -1152,16 +1157,16 @@
     </row>
     <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>10</v>
@@ -1172,16 +1177,16 @@
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>10</v>
@@ -1192,16 +1197,16 @@
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>10</v>
@@ -1212,16 +1217,16 @@
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>10</v>
@@ -1232,16 +1237,16 @@
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>10</v>
@@ -1252,16 +1257,16 @@
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>10</v>
@@ -1272,16 +1277,16 @@
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>10</v>
@@ -1292,16 +1297,16 @@
     </row>
     <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>10</v>
@@ -1312,16 +1317,16 @@
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>10</v>
@@ -1332,16 +1337,16 @@
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>10</v>
@@ -1352,16 +1357,16 @@
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>10</v>
@@ -1372,216 +1377,216 @@
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>10</v>
@@ -1592,16 +1597,16 @@
     </row>
     <row r="33" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>10</v>
@@ -1612,16 +1617,16 @@
     </row>
     <row r="34" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>10</v>
@@ -1632,16 +1637,16 @@
     </row>
     <row r="35" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>10</v>
@@ -1652,16 +1657,16 @@
     </row>
     <row r="36" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>10</v>
@@ -1672,16 +1677,16 @@
     </row>
     <row r="37" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>10</v>
@@ -1692,16 +1697,16 @@
     </row>
     <row r="38" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>10</v>
@@ -1712,16 +1717,16 @@
     </row>
     <row r="39" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>10</v>
@@ -1732,16 +1737,16 @@
     </row>
     <row r="40" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>10</v>
@@ -1752,16 +1757,16 @@
     </row>
     <row r="41" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>10</v>
@@ -1772,16 +1777,16 @@
     </row>
     <row r="42" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>10</v>
@@ -1792,16 +1797,16 @@
     </row>
     <row r="43" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>10</v>
@@ -1812,16 +1817,16 @@
     </row>
     <row r="44" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>10</v>
@@ -1832,16 +1837,16 @@
     </row>
     <row r="45" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>10</v>
@@ -1852,16 +1857,16 @@
     </row>
     <row r="46" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>10</v>
@@ -1872,16 +1877,16 @@
     </row>
     <row r="47" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>10</v>
@@ -1892,16 +1897,16 @@
     </row>
     <row r="48" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>10</v>
@@ -1912,16 +1917,16 @@
     </row>
     <row r="49" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>10</v>
@@ -1932,16 +1937,16 @@
     </row>
     <row r="50" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>10</v>
@@ -1952,16 +1957,16 @@
     </row>
     <row r="51" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>10</v>

</xml_diff>